<commit_message>
Make Monthly Report row-number formula engine-agnostic
Replace the SUMPRODUCT(--(range<>"")) sequence counter with a simpler
ROW()-based form that is equivalent given contiguous employee IDs and
evaluates correctly in every spreadsheet engine.

Co-authored-by: ayoubdexx <220752352+ayoubdexx@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Payroll_Management_System.xlsx
+++ b/Payroll_Management_System.xlsx
@@ -25482,7 +25482,7 @@
     </row>
     <row r="4">
       <c r="A4" s="58">
-        <f>IF($B4="","",SUMPRODUCT(--($B$4:$B4&lt;&gt;"")))</f>
+        <f>IF($B4="","",ROW()-4+1)</f>
       </c>
       <c r="B4" s="17">
         <f>IF('Daily Attendance'!A5="","",'Daily Attendance'!A5)</f>
@@ -25517,7 +25517,7 @@
     </row>
     <row r="5">
       <c r="A5" s="58">
-        <f>IF($B5="","",SUMPRODUCT(--($B$4:$B5&lt;&gt;"")))</f>
+        <f>IF($B5="","",ROW()-4+1)</f>
       </c>
       <c r="B5" s="17">
         <f>IF('Daily Attendance'!A6="","",'Daily Attendance'!A6)</f>
@@ -25552,7 +25552,7 @@
     </row>
     <row r="6">
       <c r="A6" s="58">
-        <f>IF($B6="","",SUMPRODUCT(--($B$4:$B6&lt;&gt;"")))</f>
+        <f>IF($B6="","",ROW()-4+1)</f>
       </c>
       <c r="B6" s="17">
         <f>IF('Daily Attendance'!A7="","",'Daily Attendance'!A7)</f>
@@ -25587,7 +25587,7 @@
     </row>
     <row r="7">
       <c r="A7" s="58">
-        <f>IF($B7="","",SUMPRODUCT(--($B$4:$B7&lt;&gt;"")))</f>
+        <f>IF($B7="","",ROW()-4+1)</f>
       </c>
       <c r="B7" s="17">
         <f>IF('Daily Attendance'!A8="","",'Daily Attendance'!A8)</f>
@@ -25622,7 +25622,7 @@
     </row>
     <row r="8">
       <c r="A8" s="58">
-        <f>IF($B8="","",SUMPRODUCT(--($B$4:$B8&lt;&gt;"")))</f>
+        <f>IF($B8="","",ROW()-4+1)</f>
       </c>
       <c r="B8" s="17">
         <f>IF('Daily Attendance'!A9="","",'Daily Attendance'!A9)</f>
@@ -25657,7 +25657,7 @@
     </row>
     <row r="9">
       <c r="A9" s="58">
-        <f>IF($B9="","",SUMPRODUCT(--($B$4:$B9&lt;&gt;"")))</f>
+        <f>IF($B9="","",ROW()-4+1)</f>
       </c>
       <c r="B9" s="17">
         <f>IF('Daily Attendance'!A10="","",'Daily Attendance'!A10)</f>
@@ -25692,7 +25692,7 @@
     </row>
     <row r="10">
       <c r="A10" s="58">
-        <f>IF($B10="","",SUMPRODUCT(--($B$4:$B10&lt;&gt;"")))</f>
+        <f>IF($B10="","",ROW()-4+1)</f>
       </c>
       <c r="B10" s="17">
         <f>IF('Daily Attendance'!A11="","",'Daily Attendance'!A11)</f>
@@ -25727,7 +25727,7 @@
     </row>
     <row r="11">
       <c r="A11" s="58">
-        <f>IF($B11="","",SUMPRODUCT(--($B$4:$B11&lt;&gt;"")))</f>
+        <f>IF($B11="","",ROW()-4+1)</f>
       </c>
       <c r="B11" s="17">
         <f>IF('Daily Attendance'!A12="","",'Daily Attendance'!A12)</f>
@@ -25762,7 +25762,7 @@
     </row>
     <row r="12">
       <c r="A12" s="58">
-        <f>IF($B12="","",SUMPRODUCT(--($B$4:$B12&lt;&gt;"")))</f>
+        <f>IF($B12="","",ROW()-4+1)</f>
       </c>
       <c r="B12" s="17">
         <f>IF('Daily Attendance'!A13="","",'Daily Attendance'!A13)</f>
@@ -25797,7 +25797,7 @@
     </row>
     <row r="13">
       <c r="A13" s="58">
-        <f>IF($B13="","",SUMPRODUCT(--($B$4:$B13&lt;&gt;"")))</f>
+        <f>IF($B13="","",ROW()-4+1)</f>
       </c>
       <c r="B13" s="17">
         <f>IF('Daily Attendance'!A14="","",'Daily Attendance'!A14)</f>
@@ -25832,7 +25832,7 @@
     </row>
     <row r="14">
       <c r="A14" s="58">
-        <f>IF($B14="","",SUMPRODUCT(--($B$4:$B14&lt;&gt;"")))</f>
+        <f>IF($B14="","",ROW()-4+1)</f>
       </c>
       <c r="B14" s="17">
         <f>IF('Daily Attendance'!A15="","",'Daily Attendance'!A15)</f>
@@ -25867,7 +25867,7 @@
     </row>
     <row r="15">
       <c r="A15" s="58">
-        <f>IF($B15="","",SUMPRODUCT(--($B$4:$B15&lt;&gt;"")))</f>
+        <f>IF($B15="","",ROW()-4+1)</f>
       </c>
       <c r="B15" s="17">
         <f>IF('Daily Attendance'!A16="","",'Daily Attendance'!A16)</f>
@@ -25902,7 +25902,7 @@
     </row>
     <row r="16">
       <c r="A16" s="58">
-        <f>IF($B16="","",SUMPRODUCT(--($B$4:$B16&lt;&gt;"")))</f>
+        <f>IF($B16="","",ROW()-4+1)</f>
       </c>
       <c r="B16" s="17">
         <f>IF('Daily Attendance'!A17="","",'Daily Attendance'!A17)</f>
@@ -25937,7 +25937,7 @@
     </row>
     <row r="17">
       <c r="A17" s="58">
-        <f>IF($B17="","",SUMPRODUCT(--($B$4:$B17&lt;&gt;"")))</f>
+        <f>IF($B17="","",ROW()-4+1)</f>
       </c>
       <c r="B17" s="17">
         <f>IF('Daily Attendance'!A18="","",'Daily Attendance'!A18)</f>
@@ -25972,7 +25972,7 @@
     </row>
     <row r="18">
       <c r="A18" s="58">
-        <f>IF($B18="","",SUMPRODUCT(--($B$4:$B18&lt;&gt;"")))</f>
+        <f>IF($B18="","",ROW()-4+1)</f>
       </c>
       <c r="B18" s="17">
         <f>IF('Daily Attendance'!A19="","",'Daily Attendance'!A19)</f>
@@ -26007,7 +26007,7 @@
     </row>
     <row r="19">
       <c r="A19" s="58">
-        <f>IF($B19="","",SUMPRODUCT(--($B$4:$B19&lt;&gt;"")))</f>
+        <f>IF($B19="","",ROW()-4+1)</f>
       </c>
       <c r="B19" s="17">
         <f>IF('Daily Attendance'!A20="","",'Daily Attendance'!A20)</f>
@@ -26042,7 +26042,7 @@
     </row>
     <row r="20">
       <c r="A20" s="58">
-        <f>IF($B20="","",SUMPRODUCT(--($B$4:$B20&lt;&gt;"")))</f>
+        <f>IF($B20="","",ROW()-4+1)</f>
       </c>
       <c r="B20" s="17">
         <f>IF('Daily Attendance'!A21="","",'Daily Attendance'!A21)</f>
@@ -26077,7 +26077,7 @@
     </row>
     <row r="21">
       <c r="A21" s="58">
-        <f>IF($B21="","",SUMPRODUCT(--($B$4:$B21&lt;&gt;"")))</f>
+        <f>IF($B21="","",ROW()-4+1)</f>
       </c>
       <c r="B21" s="17">
         <f>IF('Daily Attendance'!A22="","",'Daily Attendance'!A22)</f>
@@ -26112,7 +26112,7 @@
     </row>
     <row r="22">
       <c r="A22" s="58">
-        <f>IF($B22="","",SUMPRODUCT(--($B$4:$B22&lt;&gt;"")))</f>
+        <f>IF($B22="","",ROW()-4+1)</f>
       </c>
       <c r="B22" s="17">
         <f>IF('Daily Attendance'!A23="","",'Daily Attendance'!A23)</f>
@@ -26147,7 +26147,7 @@
     </row>
     <row r="23">
       <c r="A23" s="58">
-        <f>IF($B23="","",SUMPRODUCT(--($B$4:$B23&lt;&gt;"")))</f>
+        <f>IF($B23="","",ROW()-4+1)</f>
       </c>
       <c r="B23" s="17">
         <f>IF('Daily Attendance'!A24="","",'Daily Attendance'!A24)</f>
@@ -26182,7 +26182,7 @@
     </row>
     <row r="24">
       <c r="A24" s="58">
-        <f>IF($B24="","",SUMPRODUCT(--($B$4:$B24&lt;&gt;"")))</f>
+        <f>IF($B24="","",ROW()-4+1)</f>
       </c>
       <c r="B24" s="17">
         <f>IF('Daily Attendance'!A25="","",'Daily Attendance'!A25)</f>
@@ -26217,7 +26217,7 @@
     </row>
     <row r="25">
       <c r="A25" s="58">
-        <f>IF($B25="","",SUMPRODUCT(--($B$4:$B25&lt;&gt;"")))</f>
+        <f>IF($B25="","",ROW()-4+1)</f>
       </c>
       <c r="B25" s="17">
         <f>IF('Daily Attendance'!A26="","",'Daily Attendance'!A26)</f>
@@ -26252,7 +26252,7 @@
     </row>
     <row r="26">
       <c r="A26" s="58">
-        <f>IF($B26="","",SUMPRODUCT(--($B$4:$B26&lt;&gt;"")))</f>
+        <f>IF($B26="","",ROW()-4+1)</f>
       </c>
       <c r="B26" s="17">
         <f>IF('Daily Attendance'!A27="","",'Daily Attendance'!A27)</f>
@@ -26287,7 +26287,7 @@
     </row>
     <row r="27">
       <c r="A27" s="58">
-        <f>IF($B27="","",SUMPRODUCT(--($B$4:$B27&lt;&gt;"")))</f>
+        <f>IF($B27="","",ROW()-4+1)</f>
       </c>
       <c r="B27" s="17">
         <f>IF('Daily Attendance'!A28="","",'Daily Attendance'!A28)</f>
@@ -26322,7 +26322,7 @@
     </row>
     <row r="28">
       <c r="A28" s="58">
-        <f>IF($B28="","",SUMPRODUCT(--($B$4:$B28&lt;&gt;"")))</f>
+        <f>IF($B28="","",ROW()-4+1)</f>
       </c>
       <c r="B28" s="17">
         <f>IF('Daily Attendance'!A29="","",'Daily Attendance'!A29)</f>
@@ -26357,7 +26357,7 @@
     </row>
     <row r="29">
       <c r="A29" s="58">
-        <f>IF($B29="","",SUMPRODUCT(--($B$4:$B29&lt;&gt;"")))</f>
+        <f>IF($B29="","",ROW()-4+1)</f>
       </c>
       <c r="B29" s="17">
         <f>IF('Daily Attendance'!A30="","",'Daily Attendance'!A30)</f>
@@ -26392,7 +26392,7 @@
     </row>
     <row r="30">
       <c r="A30" s="58">
-        <f>IF($B30="","",SUMPRODUCT(--($B$4:$B30&lt;&gt;"")))</f>
+        <f>IF($B30="","",ROW()-4+1)</f>
       </c>
       <c r="B30" s="17">
         <f>IF('Daily Attendance'!A31="","",'Daily Attendance'!A31)</f>
@@ -26427,7 +26427,7 @@
     </row>
     <row r="31">
       <c r="A31" s="58">
-        <f>IF($B31="","",SUMPRODUCT(--($B$4:$B31&lt;&gt;"")))</f>
+        <f>IF($B31="","",ROW()-4+1)</f>
       </c>
       <c r="B31" s="17">
         <f>IF('Daily Attendance'!A32="","",'Daily Attendance'!A32)</f>
@@ -26462,7 +26462,7 @@
     </row>
     <row r="32">
       <c r="A32" s="58">
-        <f>IF($B32="","",SUMPRODUCT(--($B$4:$B32&lt;&gt;"")))</f>
+        <f>IF($B32="","",ROW()-4+1)</f>
       </c>
       <c r="B32" s="17">
         <f>IF('Daily Attendance'!A33="","",'Daily Attendance'!A33)</f>
@@ -26497,7 +26497,7 @@
     </row>
     <row r="33">
       <c r="A33" s="58">
-        <f>IF($B33="","",SUMPRODUCT(--($B$4:$B33&lt;&gt;"")))</f>
+        <f>IF($B33="","",ROW()-4+1)</f>
       </c>
       <c r="B33" s="17">
         <f>IF('Daily Attendance'!A34="","",'Daily Attendance'!A34)</f>
@@ -26532,7 +26532,7 @@
     </row>
     <row r="34">
       <c r="A34" s="58">
-        <f>IF($B34="","",SUMPRODUCT(--($B$4:$B34&lt;&gt;"")))</f>
+        <f>IF($B34="","",ROW()-4+1)</f>
       </c>
       <c r="B34" s="17">
         <f>IF('Daily Attendance'!A35="","",'Daily Attendance'!A35)</f>
@@ -26567,7 +26567,7 @@
     </row>
     <row r="35">
       <c r="A35" s="58">
-        <f>IF($B35="","",SUMPRODUCT(--($B$4:$B35&lt;&gt;"")))</f>
+        <f>IF($B35="","",ROW()-4+1)</f>
       </c>
       <c r="B35" s="17">
         <f>IF('Daily Attendance'!A36="","",'Daily Attendance'!A36)</f>
@@ -26602,7 +26602,7 @@
     </row>
     <row r="36">
       <c r="A36" s="58">
-        <f>IF($B36="","",SUMPRODUCT(--($B$4:$B36&lt;&gt;"")))</f>
+        <f>IF($B36="","",ROW()-4+1)</f>
       </c>
       <c r="B36" s="17">
         <f>IF('Daily Attendance'!A37="","",'Daily Attendance'!A37)</f>
@@ -26637,7 +26637,7 @@
     </row>
     <row r="37">
       <c r="A37" s="58">
-        <f>IF($B37="","",SUMPRODUCT(--($B$4:$B37&lt;&gt;"")))</f>
+        <f>IF($B37="","",ROW()-4+1)</f>
       </c>
       <c r="B37" s="17">
         <f>IF('Daily Attendance'!A38="","",'Daily Attendance'!A38)</f>
@@ -26672,7 +26672,7 @@
     </row>
     <row r="38">
       <c r="A38" s="58">
-        <f>IF($B38="","",SUMPRODUCT(--($B$4:$B38&lt;&gt;"")))</f>
+        <f>IF($B38="","",ROW()-4+1)</f>
       </c>
       <c r="B38" s="17">
         <f>IF('Daily Attendance'!A39="","",'Daily Attendance'!A39)</f>
@@ -26707,7 +26707,7 @@
     </row>
     <row r="39">
       <c r="A39" s="58">
-        <f>IF($B39="","",SUMPRODUCT(--($B$4:$B39&lt;&gt;"")))</f>
+        <f>IF($B39="","",ROW()-4+1)</f>
       </c>
       <c r="B39" s="17">
         <f>IF('Daily Attendance'!A40="","",'Daily Attendance'!A40)</f>
@@ -26742,7 +26742,7 @@
     </row>
     <row r="40">
       <c r="A40" s="58">
-        <f>IF($B40="","",SUMPRODUCT(--($B$4:$B40&lt;&gt;"")))</f>
+        <f>IF($B40="","",ROW()-4+1)</f>
       </c>
       <c r="B40" s="17">
         <f>IF('Daily Attendance'!A41="","",'Daily Attendance'!A41)</f>
@@ -26777,7 +26777,7 @@
     </row>
     <row r="41">
       <c r="A41" s="58">
-        <f>IF($B41="","",SUMPRODUCT(--($B$4:$B41&lt;&gt;"")))</f>
+        <f>IF($B41="","",ROW()-4+1)</f>
       </c>
       <c r="B41" s="17">
         <f>IF('Daily Attendance'!A42="","",'Daily Attendance'!A42)</f>
@@ -26812,7 +26812,7 @@
     </row>
     <row r="42">
       <c r="A42" s="58">
-        <f>IF($B42="","",SUMPRODUCT(--($B$4:$B42&lt;&gt;"")))</f>
+        <f>IF($B42="","",ROW()-4+1)</f>
       </c>
       <c r="B42" s="17">
         <f>IF('Daily Attendance'!A43="","",'Daily Attendance'!A43)</f>
@@ -26847,7 +26847,7 @@
     </row>
     <row r="43">
       <c r="A43" s="58">
-        <f>IF($B43="","",SUMPRODUCT(--($B$4:$B43&lt;&gt;"")))</f>
+        <f>IF($B43="","",ROW()-4+1)</f>
       </c>
       <c r="B43" s="17">
         <f>IF('Daily Attendance'!A44="","",'Daily Attendance'!A44)</f>
@@ -26882,7 +26882,7 @@
     </row>
     <row r="44">
       <c r="A44" s="58">
-        <f>IF($B44="","",SUMPRODUCT(--($B$4:$B44&lt;&gt;"")))</f>
+        <f>IF($B44="","",ROW()-4+1)</f>
       </c>
       <c r="B44" s="17">
         <f>IF('Daily Attendance'!A45="","",'Daily Attendance'!A45)</f>
@@ -26917,7 +26917,7 @@
     </row>
     <row r="45">
       <c r="A45" s="58">
-        <f>IF($B45="","",SUMPRODUCT(--($B$4:$B45&lt;&gt;"")))</f>
+        <f>IF($B45="","",ROW()-4+1)</f>
       </c>
       <c r="B45" s="17">
         <f>IF('Daily Attendance'!A46="","",'Daily Attendance'!A46)</f>
@@ -26952,7 +26952,7 @@
     </row>
     <row r="46">
       <c r="A46" s="58">
-        <f>IF($B46="","",SUMPRODUCT(--($B$4:$B46&lt;&gt;"")))</f>
+        <f>IF($B46="","",ROW()-4+1)</f>
       </c>
       <c r="B46" s="17">
         <f>IF('Daily Attendance'!A47="","",'Daily Attendance'!A47)</f>
@@ -26987,7 +26987,7 @@
     </row>
     <row r="47">
       <c r="A47" s="58">
-        <f>IF($B47="","",SUMPRODUCT(--($B$4:$B47&lt;&gt;"")))</f>
+        <f>IF($B47="","",ROW()-4+1)</f>
       </c>
       <c r="B47" s="17">
         <f>IF('Daily Attendance'!A48="","",'Daily Attendance'!A48)</f>
@@ -27022,7 +27022,7 @@
     </row>
     <row r="48">
       <c r="A48" s="58">
-        <f>IF($B48="","",SUMPRODUCT(--($B$4:$B48&lt;&gt;"")))</f>
+        <f>IF($B48="","",ROW()-4+1)</f>
       </c>
       <c r="B48" s="17">
         <f>IF('Daily Attendance'!A49="","",'Daily Attendance'!A49)</f>
@@ -27057,7 +27057,7 @@
     </row>
     <row r="49">
       <c r="A49" s="58">
-        <f>IF($B49="","",SUMPRODUCT(--($B$4:$B49&lt;&gt;"")))</f>
+        <f>IF($B49="","",ROW()-4+1)</f>
       </c>
       <c r="B49" s="17">
         <f>IF('Daily Attendance'!A50="","",'Daily Attendance'!A50)</f>
@@ -27092,7 +27092,7 @@
     </row>
     <row r="50">
       <c r="A50" s="58">
-        <f>IF($B50="","",SUMPRODUCT(--($B$4:$B50&lt;&gt;"")))</f>
+        <f>IF($B50="","",ROW()-4+1)</f>
       </c>
       <c r="B50" s="17">
         <f>IF('Daily Attendance'!A51="","",'Daily Attendance'!A51)</f>
@@ -27127,7 +27127,7 @@
     </row>
     <row r="51">
       <c r="A51" s="58">
-        <f>IF($B51="","",SUMPRODUCT(--($B$4:$B51&lt;&gt;"")))</f>
+        <f>IF($B51="","",ROW()-4+1)</f>
       </c>
       <c r="B51" s="17">
         <f>IF('Daily Attendance'!A52="","",'Daily Attendance'!A52)</f>
@@ -27162,7 +27162,7 @@
     </row>
     <row r="52">
       <c r="A52" s="58">
-        <f>IF($B52="","",SUMPRODUCT(--($B$4:$B52&lt;&gt;"")))</f>
+        <f>IF($B52="","",ROW()-4+1)</f>
       </c>
       <c r="B52" s="17">
         <f>IF('Daily Attendance'!A53="","",'Daily Attendance'!A53)</f>
@@ -27197,7 +27197,7 @@
     </row>
     <row r="53">
       <c r="A53" s="58">
-        <f>IF($B53="","",SUMPRODUCT(--($B$4:$B53&lt;&gt;"")))</f>
+        <f>IF($B53="","",ROW()-4+1)</f>
       </c>
       <c r="B53" s="17">
         <f>IF('Daily Attendance'!A54="","",'Daily Attendance'!A54)</f>
@@ -27232,7 +27232,7 @@
     </row>
     <row r="54">
       <c r="A54" s="58">
-        <f>IF($B54="","",SUMPRODUCT(--($B$4:$B54&lt;&gt;"")))</f>
+        <f>IF($B54="","",ROW()-4+1)</f>
       </c>
       <c r="B54" s="17">
         <f>IF('Daily Attendance'!A55="","",'Daily Attendance'!A55)</f>
@@ -27267,7 +27267,7 @@
     </row>
     <row r="55">
       <c r="A55" s="58">
-        <f>IF($B55="","",SUMPRODUCT(--($B$4:$B55&lt;&gt;"")))</f>
+        <f>IF($B55="","",ROW()-4+1)</f>
       </c>
       <c r="B55" s="17">
         <f>IF('Daily Attendance'!A56="","",'Daily Attendance'!A56)</f>
@@ -27302,7 +27302,7 @@
     </row>
     <row r="56">
       <c r="A56" s="58">
-        <f>IF($B56="","",SUMPRODUCT(--($B$4:$B56&lt;&gt;"")))</f>
+        <f>IF($B56="","",ROW()-4+1)</f>
       </c>
       <c r="B56" s="17">
         <f>IF('Daily Attendance'!A57="","",'Daily Attendance'!A57)</f>
@@ -27337,7 +27337,7 @@
     </row>
     <row r="57">
       <c r="A57" s="58">
-        <f>IF($B57="","",SUMPRODUCT(--($B$4:$B57&lt;&gt;"")))</f>
+        <f>IF($B57="","",ROW()-4+1)</f>
       </c>
       <c r="B57" s="17">
         <f>IF('Daily Attendance'!A58="","",'Daily Attendance'!A58)</f>
@@ -27372,7 +27372,7 @@
     </row>
     <row r="58">
       <c r="A58" s="58">
-        <f>IF($B58="","",SUMPRODUCT(--($B$4:$B58&lt;&gt;"")))</f>
+        <f>IF($B58="","",ROW()-4+1)</f>
       </c>
       <c r="B58" s="17">
         <f>IF('Daily Attendance'!A59="","",'Daily Attendance'!A59)</f>
@@ -27407,7 +27407,7 @@
     </row>
     <row r="59">
       <c r="A59" s="58">
-        <f>IF($B59="","",SUMPRODUCT(--($B$4:$B59&lt;&gt;"")))</f>
+        <f>IF($B59="","",ROW()-4+1)</f>
       </c>
       <c r="B59" s="17">
         <f>IF('Daily Attendance'!A60="","",'Daily Attendance'!A60)</f>
@@ -27442,7 +27442,7 @@
     </row>
     <row r="60">
       <c r="A60" s="58">
-        <f>IF($B60="","",SUMPRODUCT(--($B$4:$B60&lt;&gt;"")))</f>
+        <f>IF($B60="","",ROW()-4+1)</f>
       </c>
       <c r="B60" s="17">
         <f>IF('Daily Attendance'!A61="","",'Daily Attendance'!A61)</f>
@@ -27477,7 +27477,7 @@
     </row>
     <row r="61">
       <c r="A61" s="58">
-        <f>IF($B61="","",SUMPRODUCT(--($B$4:$B61&lt;&gt;"")))</f>
+        <f>IF($B61="","",ROW()-4+1)</f>
       </c>
       <c r="B61" s="17">
         <f>IF('Daily Attendance'!A62="","",'Daily Attendance'!A62)</f>
@@ -27512,7 +27512,7 @@
     </row>
     <row r="62">
       <c r="A62" s="58">
-        <f>IF($B62="","",SUMPRODUCT(--($B$4:$B62&lt;&gt;"")))</f>
+        <f>IF($B62="","",ROW()-4+1)</f>
       </c>
       <c r="B62" s="17">
         <f>IF('Daily Attendance'!A63="","",'Daily Attendance'!A63)</f>
@@ -27547,7 +27547,7 @@
     </row>
     <row r="63">
       <c r="A63" s="58">
-        <f>IF($B63="","",SUMPRODUCT(--($B$4:$B63&lt;&gt;"")))</f>
+        <f>IF($B63="","",ROW()-4+1)</f>
       </c>
       <c r="B63" s="17">
         <f>IF('Daily Attendance'!A64="","",'Daily Attendance'!A64)</f>
@@ -27582,7 +27582,7 @@
     </row>
     <row r="64">
       <c r="A64" s="58">
-        <f>IF($B64="","",SUMPRODUCT(--($B$4:$B64&lt;&gt;"")))</f>
+        <f>IF($B64="","",ROW()-4+1)</f>
       </c>
       <c r="B64" s="17">
         <f>IF('Daily Attendance'!A65="","",'Daily Attendance'!A65)</f>
@@ -27617,7 +27617,7 @@
     </row>
     <row r="65">
       <c r="A65" s="58">
-        <f>IF($B65="","",SUMPRODUCT(--($B$4:$B65&lt;&gt;"")))</f>
+        <f>IF($B65="","",ROW()-4+1)</f>
       </c>
       <c r="B65" s="17">
         <f>IF('Daily Attendance'!A66="","",'Daily Attendance'!A66)</f>
@@ -27652,7 +27652,7 @@
     </row>
     <row r="66">
       <c r="A66" s="58">
-        <f>IF($B66="","",SUMPRODUCT(--($B$4:$B66&lt;&gt;"")))</f>
+        <f>IF($B66="","",ROW()-4+1)</f>
       </c>
       <c r="B66" s="17">
         <f>IF('Daily Attendance'!A67="","",'Daily Attendance'!A67)</f>
@@ -27687,7 +27687,7 @@
     </row>
     <row r="67">
       <c r="A67" s="58">
-        <f>IF($B67="","",SUMPRODUCT(--($B$4:$B67&lt;&gt;"")))</f>
+        <f>IF($B67="","",ROW()-4+1)</f>
       </c>
       <c r="B67" s="17">
         <f>IF('Daily Attendance'!A68="","",'Daily Attendance'!A68)</f>
@@ -27722,7 +27722,7 @@
     </row>
     <row r="68">
       <c r="A68" s="58">
-        <f>IF($B68="","",SUMPRODUCT(--($B$4:$B68&lt;&gt;"")))</f>
+        <f>IF($B68="","",ROW()-4+1)</f>
       </c>
       <c r="B68" s="17">
         <f>IF('Daily Attendance'!A69="","",'Daily Attendance'!A69)</f>
@@ -27757,7 +27757,7 @@
     </row>
     <row r="69">
       <c r="A69" s="58">
-        <f>IF($B69="","",SUMPRODUCT(--($B$4:$B69&lt;&gt;"")))</f>
+        <f>IF($B69="","",ROW()-4+1)</f>
       </c>
       <c r="B69" s="17">
         <f>IF('Daily Attendance'!A70="","",'Daily Attendance'!A70)</f>
@@ -27792,7 +27792,7 @@
     </row>
     <row r="70">
       <c r="A70" s="58">
-        <f>IF($B70="","",SUMPRODUCT(--($B$4:$B70&lt;&gt;"")))</f>
+        <f>IF($B70="","",ROW()-4+1)</f>
       </c>
       <c r="B70" s="17">
         <f>IF('Daily Attendance'!A71="","",'Daily Attendance'!A71)</f>
@@ -27827,7 +27827,7 @@
     </row>
     <row r="71">
       <c r="A71" s="58">
-        <f>IF($B71="","",SUMPRODUCT(--($B$4:$B71&lt;&gt;"")))</f>
+        <f>IF($B71="","",ROW()-4+1)</f>
       </c>
       <c r="B71" s="17">
         <f>IF('Daily Attendance'!A72="","",'Daily Attendance'!A72)</f>
@@ -27862,7 +27862,7 @@
     </row>
     <row r="72">
       <c r="A72" s="58">
-        <f>IF($B72="","",SUMPRODUCT(--($B$4:$B72&lt;&gt;"")))</f>
+        <f>IF($B72="","",ROW()-4+1)</f>
       </c>
       <c r="B72" s="17">
         <f>IF('Daily Attendance'!A73="","",'Daily Attendance'!A73)</f>
@@ -27897,7 +27897,7 @@
     </row>
     <row r="73">
       <c r="A73" s="58">
-        <f>IF($B73="","",SUMPRODUCT(--($B$4:$B73&lt;&gt;"")))</f>
+        <f>IF($B73="","",ROW()-4+1)</f>
       </c>
       <c r="B73" s="17">
         <f>IF('Daily Attendance'!A74="","",'Daily Attendance'!A74)</f>
@@ -27932,7 +27932,7 @@
     </row>
     <row r="74">
       <c r="A74" s="58">
-        <f>IF($B74="","",SUMPRODUCT(--($B$4:$B74&lt;&gt;"")))</f>
+        <f>IF($B74="","",ROW()-4+1)</f>
       </c>
       <c r="B74" s="17">
         <f>IF('Daily Attendance'!A75="","",'Daily Attendance'!A75)</f>
@@ -27967,7 +27967,7 @@
     </row>
     <row r="75">
       <c r="A75" s="58">
-        <f>IF($B75="","",SUMPRODUCT(--($B$4:$B75&lt;&gt;"")))</f>
+        <f>IF($B75="","",ROW()-4+1)</f>
       </c>
       <c r="B75" s="17">
         <f>IF('Daily Attendance'!A76="","",'Daily Attendance'!A76)</f>
@@ -28002,7 +28002,7 @@
     </row>
     <row r="76">
       <c r="A76" s="58">
-        <f>IF($B76="","",SUMPRODUCT(--($B$4:$B76&lt;&gt;"")))</f>
+        <f>IF($B76="","",ROW()-4+1)</f>
       </c>
       <c r="B76" s="17">
         <f>IF('Daily Attendance'!A77="","",'Daily Attendance'!A77)</f>
@@ -28037,7 +28037,7 @@
     </row>
     <row r="77">
       <c r="A77" s="58">
-        <f>IF($B77="","",SUMPRODUCT(--($B$4:$B77&lt;&gt;"")))</f>
+        <f>IF($B77="","",ROW()-4+1)</f>
       </c>
       <c r="B77" s="17">
         <f>IF('Daily Attendance'!A78="","",'Daily Attendance'!A78)</f>
@@ -28072,7 +28072,7 @@
     </row>
     <row r="78">
       <c r="A78" s="58">
-        <f>IF($B78="","",SUMPRODUCT(--($B$4:$B78&lt;&gt;"")))</f>
+        <f>IF($B78="","",ROW()-4+1)</f>
       </c>
       <c r="B78" s="17">
         <f>IF('Daily Attendance'!A79="","",'Daily Attendance'!A79)</f>
@@ -28107,7 +28107,7 @@
     </row>
     <row r="79">
       <c r="A79" s="58">
-        <f>IF($B79="","",SUMPRODUCT(--($B$4:$B79&lt;&gt;"")))</f>
+        <f>IF($B79="","",ROW()-4+1)</f>
       </c>
       <c r="B79" s="17">
         <f>IF('Daily Attendance'!A80="","",'Daily Attendance'!A80)</f>
@@ -28142,7 +28142,7 @@
     </row>
     <row r="80">
       <c r="A80" s="58">
-        <f>IF($B80="","",SUMPRODUCT(--($B$4:$B80&lt;&gt;"")))</f>
+        <f>IF($B80="","",ROW()-4+1)</f>
       </c>
       <c r="B80" s="17">
         <f>IF('Daily Attendance'!A81="","",'Daily Attendance'!A81)</f>
@@ -28177,7 +28177,7 @@
     </row>
     <row r="81">
       <c r="A81" s="58">
-        <f>IF($B81="","",SUMPRODUCT(--($B$4:$B81&lt;&gt;"")))</f>
+        <f>IF($B81="","",ROW()-4+1)</f>
       </c>
       <c r="B81" s="17">
         <f>IF('Daily Attendance'!A82="","",'Daily Attendance'!A82)</f>
@@ -28212,7 +28212,7 @@
     </row>
     <row r="82">
       <c r="A82" s="58">
-        <f>IF($B82="","",SUMPRODUCT(--($B$4:$B82&lt;&gt;"")))</f>
+        <f>IF($B82="","",ROW()-4+1)</f>
       </c>
       <c r="B82" s="17">
         <f>IF('Daily Attendance'!A83="","",'Daily Attendance'!A83)</f>
@@ -28247,7 +28247,7 @@
     </row>
     <row r="83">
       <c r="A83" s="58">
-        <f>IF($B83="","",SUMPRODUCT(--($B$4:$B83&lt;&gt;"")))</f>
+        <f>IF($B83="","",ROW()-4+1)</f>
       </c>
       <c r="B83" s="17">
         <f>IF('Daily Attendance'!A84="","",'Daily Attendance'!A84)</f>
@@ -28282,7 +28282,7 @@
     </row>
     <row r="84">
       <c r="A84" s="58">
-        <f>IF($B84="","",SUMPRODUCT(--($B$4:$B84&lt;&gt;"")))</f>
+        <f>IF($B84="","",ROW()-4+1)</f>
       </c>
       <c r="B84" s="17">
         <f>IF('Daily Attendance'!A85="","",'Daily Attendance'!A85)</f>
@@ -28317,7 +28317,7 @@
     </row>
     <row r="85">
       <c r="A85" s="58">
-        <f>IF($B85="","",SUMPRODUCT(--($B$4:$B85&lt;&gt;"")))</f>
+        <f>IF($B85="","",ROW()-4+1)</f>
       </c>
       <c r="B85" s="17">
         <f>IF('Daily Attendance'!A86="","",'Daily Attendance'!A86)</f>
@@ -28352,7 +28352,7 @@
     </row>
     <row r="86">
       <c r="A86" s="58">
-        <f>IF($B86="","",SUMPRODUCT(--($B$4:$B86&lt;&gt;"")))</f>
+        <f>IF($B86="","",ROW()-4+1)</f>
       </c>
       <c r="B86" s="17">
         <f>IF('Daily Attendance'!A87="","",'Daily Attendance'!A87)</f>
@@ -28387,7 +28387,7 @@
     </row>
     <row r="87">
       <c r="A87" s="58">
-        <f>IF($B87="","",SUMPRODUCT(--($B$4:$B87&lt;&gt;"")))</f>
+        <f>IF($B87="","",ROW()-4+1)</f>
       </c>
       <c r="B87" s="17">
         <f>IF('Daily Attendance'!A88="","",'Daily Attendance'!A88)</f>
@@ -28422,7 +28422,7 @@
     </row>
     <row r="88">
       <c r="A88" s="58">
-        <f>IF($B88="","",SUMPRODUCT(--($B$4:$B88&lt;&gt;"")))</f>
+        <f>IF($B88="","",ROW()-4+1)</f>
       </c>
       <c r="B88" s="17">
         <f>IF('Daily Attendance'!A89="","",'Daily Attendance'!A89)</f>
@@ -28457,7 +28457,7 @@
     </row>
     <row r="89">
       <c r="A89" s="58">
-        <f>IF($B89="","",SUMPRODUCT(--($B$4:$B89&lt;&gt;"")))</f>
+        <f>IF($B89="","",ROW()-4+1)</f>
       </c>
       <c r="B89" s="17">
         <f>IF('Daily Attendance'!A90="","",'Daily Attendance'!A90)</f>
@@ -28492,7 +28492,7 @@
     </row>
     <row r="90">
       <c r="A90" s="58">
-        <f>IF($B90="","",SUMPRODUCT(--($B$4:$B90&lt;&gt;"")))</f>
+        <f>IF($B90="","",ROW()-4+1)</f>
       </c>
       <c r="B90" s="17">
         <f>IF('Daily Attendance'!A91="","",'Daily Attendance'!A91)</f>
@@ -28527,7 +28527,7 @@
     </row>
     <row r="91">
       <c r="A91" s="58">
-        <f>IF($B91="","",SUMPRODUCT(--($B$4:$B91&lt;&gt;"")))</f>
+        <f>IF($B91="","",ROW()-4+1)</f>
       </c>
       <c r="B91" s="17">
         <f>IF('Daily Attendance'!A92="","",'Daily Attendance'!A92)</f>
@@ -28562,7 +28562,7 @@
     </row>
     <row r="92">
       <c r="A92" s="58">
-        <f>IF($B92="","",SUMPRODUCT(--($B$4:$B92&lt;&gt;"")))</f>
+        <f>IF($B92="","",ROW()-4+1)</f>
       </c>
       <c r="B92" s="17">
         <f>IF('Daily Attendance'!A93="","",'Daily Attendance'!A93)</f>
@@ -28597,7 +28597,7 @@
     </row>
     <row r="93">
       <c r="A93" s="58">
-        <f>IF($B93="","",SUMPRODUCT(--($B$4:$B93&lt;&gt;"")))</f>
+        <f>IF($B93="","",ROW()-4+1)</f>
       </c>
       <c r="B93" s="17">
         <f>IF('Daily Attendance'!A94="","",'Daily Attendance'!A94)</f>
@@ -28632,7 +28632,7 @@
     </row>
     <row r="94">
       <c r="A94" s="58">
-        <f>IF($B94="","",SUMPRODUCT(--($B$4:$B94&lt;&gt;"")))</f>
+        <f>IF($B94="","",ROW()-4+1)</f>
       </c>
       <c r="B94" s="17">
         <f>IF('Daily Attendance'!A95="","",'Daily Attendance'!A95)</f>
@@ -28667,7 +28667,7 @@
     </row>
     <row r="95">
       <c r="A95" s="58">
-        <f>IF($B95="","",SUMPRODUCT(--($B$4:$B95&lt;&gt;"")))</f>
+        <f>IF($B95="","",ROW()-4+1)</f>
       </c>
       <c r="B95" s="17">
         <f>IF('Daily Attendance'!A96="","",'Daily Attendance'!A96)</f>
@@ -28702,7 +28702,7 @@
     </row>
     <row r="96">
       <c r="A96" s="58">
-        <f>IF($B96="","",SUMPRODUCT(--($B$4:$B96&lt;&gt;"")))</f>
+        <f>IF($B96="","",ROW()-4+1)</f>
       </c>
       <c r="B96" s="17">
         <f>IF('Daily Attendance'!A97="","",'Daily Attendance'!A97)</f>
@@ -28737,7 +28737,7 @@
     </row>
     <row r="97">
       <c r="A97" s="58">
-        <f>IF($B97="","",SUMPRODUCT(--($B$4:$B97&lt;&gt;"")))</f>
+        <f>IF($B97="","",ROW()-4+1)</f>
       </c>
       <c r="B97" s="17">
         <f>IF('Daily Attendance'!A98="","",'Daily Attendance'!A98)</f>
@@ -28772,7 +28772,7 @@
     </row>
     <row r="98">
       <c r="A98" s="58">
-        <f>IF($B98="","",SUMPRODUCT(--($B$4:$B98&lt;&gt;"")))</f>
+        <f>IF($B98="","",ROW()-4+1)</f>
       </c>
       <c r="B98" s="17">
         <f>IF('Daily Attendance'!A99="","",'Daily Attendance'!A99)</f>
@@ -28807,7 +28807,7 @@
     </row>
     <row r="99">
       <c r="A99" s="58">
-        <f>IF($B99="","",SUMPRODUCT(--($B$4:$B99&lt;&gt;"")))</f>
+        <f>IF($B99="","",ROW()-4+1)</f>
       </c>
       <c r="B99" s="17">
         <f>IF('Daily Attendance'!A100="","",'Daily Attendance'!A100)</f>
@@ -28842,7 +28842,7 @@
     </row>
     <row r="100">
       <c r="A100" s="58">
-        <f>IF($B100="","",SUMPRODUCT(--($B$4:$B100&lt;&gt;"")))</f>
+        <f>IF($B100="","",ROW()-4+1)</f>
       </c>
       <c r="B100" s="17">
         <f>IF('Daily Attendance'!A101="","",'Daily Attendance'!A101)</f>
@@ -28877,7 +28877,7 @@
     </row>
     <row r="101">
       <c r="A101" s="58">
-        <f>IF($B101="","",SUMPRODUCT(--($B$4:$B101&lt;&gt;"")))</f>
+        <f>IF($B101="","",ROW()-4+1)</f>
       </c>
       <c r="B101" s="17">
         <f>IF('Daily Attendance'!A102="","",'Daily Attendance'!A102)</f>
@@ -28912,7 +28912,7 @@
     </row>
     <row r="102">
       <c r="A102" s="58">
-        <f>IF($B102="","",SUMPRODUCT(--($B$4:$B102&lt;&gt;"")))</f>
+        <f>IF($B102="","",ROW()-4+1)</f>
       </c>
       <c r="B102" s="17">
         <f>IF('Daily Attendance'!A103="","",'Daily Attendance'!A103)</f>
@@ -28947,7 +28947,7 @@
     </row>
     <row r="103">
       <c r="A103" s="58">
-        <f>IF($B103="","",SUMPRODUCT(--($B$4:$B103&lt;&gt;"")))</f>
+        <f>IF($B103="","",ROW()-4+1)</f>
       </c>
       <c r="B103" s="17">
         <f>IF('Daily Attendance'!A104="","",'Daily Attendance'!A104)</f>
@@ -28982,7 +28982,7 @@
     </row>
     <row r="104">
       <c r="A104" s="58">
-        <f>IF($B104="","",SUMPRODUCT(--($B$4:$B104&lt;&gt;"")))</f>
+        <f>IF($B104="","",ROW()-4+1)</f>
       </c>
       <c r="B104" s="17">
         <f>IF('Daily Attendance'!A105="","",'Daily Attendance'!A105)</f>
@@ -29017,7 +29017,7 @@
     </row>
     <row r="105">
       <c r="A105" s="58">
-        <f>IF($B105="","",SUMPRODUCT(--($B$4:$B105&lt;&gt;"")))</f>
+        <f>IF($B105="","",ROW()-4+1)</f>
       </c>
       <c r="B105" s="17">
         <f>IF('Daily Attendance'!A106="","",'Daily Attendance'!A106)</f>
@@ -29052,7 +29052,7 @@
     </row>
     <row r="106">
       <c r="A106" s="58">
-        <f>IF($B106="","",SUMPRODUCT(--($B$4:$B106&lt;&gt;"")))</f>
+        <f>IF($B106="","",ROW()-4+1)</f>
       </c>
       <c r="B106" s="17">
         <f>IF('Daily Attendance'!A107="","",'Daily Attendance'!A107)</f>
@@ -29087,7 +29087,7 @@
     </row>
     <row r="107">
       <c r="A107" s="58">
-        <f>IF($B107="","",SUMPRODUCT(--($B$4:$B107&lt;&gt;"")))</f>
+        <f>IF($B107="","",ROW()-4+1)</f>
       </c>
       <c r="B107" s="17">
         <f>IF('Daily Attendance'!A108="","",'Daily Attendance'!A108)</f>
@@ -29122,7 +29122,7 @@
     </row>
     <row r="108">
       <c r="A108" s="58">
-        <f>IF($B108="","",SUMPRODUCT(--($B$4:$B108&lt;&gt;"")))</f>
+        <f>IF($B108="","",ROW()-4+1)</f>
       </c>
       <c r="B108" s="17">
         <f>IF('Daily Attendance'!A109="","",'Daily Attendance'!A109)</f>
@@ -29157,7 +29157,7 @@
     </row>
     <row r="109">
       <c r="A109" s="58">
-        <f>IF($B109="","",SUMPRODUCT(--($B$4:$B109&lt;&gt;"")))</f>
+        <f>IF($B109="","",ROW()-4+1)</f>
       </c>
       <c r="B109" s="17">
         <f>IF('Daily Attendance'!A110="","",'Daily Attendance'!A110)</f>
@@ -29192,7 +29192,7 @@
     </row>
     <row r="110">
       <c r="A110" s="58">
-        <f>IF($B110="","",SUMPRODUCT(--($B$4:$B110&lt;&gt;"")))</f>
+        <f>IF($B110="","",ROW()-4+1)</f>
       </c>
       <c r="B110" s="17">
         <f>IF('Daily Attendance'!A111="","",'Daily Attendance'!A111)</f>
@@ -29227,7 +29227,7 @@
     </row>
     <row r="111">
       <c r="A111" s="58">
-        <f>IF($B111="","",SUMPRODUCT(--($B$4:$B111&lt;&gt;"")))</f>
+        <f>IF($B111="","",ROW()-4+1)</f>
       </c>
       <c r="B111" s="17">
         <f>IF('Daily Attendance'!A112="","",'Daily Attendance'!A112)</f>
@@ -29262,7 +29262,7 @@
     </row>
     <row r="112">
       <c r="A112" s="58">
-        <f>IF($B112="","",SUMPRODUCT(--($B$4:$B112&lt;&gt;"")))</f>
+        <f>IF($B112="","",ROW()-4+1)</f>
       </c>
       <c r="B112" s="17">
         <f>IF('Daily Attendance'!A113="","",'Daily Attendance'!A113)</f>
@@ -29297,7 +29297,7 @@
     </row>
     <row r="113">
       <c r="A113" s="58">
-        <f>IF($B113="","",SUMPRODUCT(--($B$4:$B113&lt;&gt;"")))</f>
+        <f>IF($B113="","",ROW()-4+1)</f>
       </c>
       <c r="B113" s="17">
         <f>IF('Daily Attendance'!A114="","",'Daily Attendance'!A114)</f>
@@ -29332,7 +29332,7 @@
     </row>
     <row r="114">
       <c r="A114" s="58">
-        <f>IF($B114="","",SUMPRODUCT(--($B$4:$B114&lt;&gt;"")))</f>
+        <f>IF($B114="","",ROW()-4+1)</f>
       </c>
       <c r="B114" s="17">
         <f>IF('Daily Attendance'!A115="","",'Daily Attendance'!A115)</f>
@@ -29367,7 +29367,7 @@
     </row>
     <row r="115">
       <c r="A115" s="58">
-        <f>IF($B115="","",SUMPRODUCT(--($B$4:$B115&lt;&gt;"")))</f>
+        <f>IF($B115="","",ROW()-4+1)</f>
       </c>
       <c r="B115" s="17">
         <f>IF('Daily Attendance'!A116="","",'Daily Attendance'!A116)</f>
@@ -29402,7 +29402,7 @@
     </row>
     <row r="116">
       <c r="A116" s="58">
-        <f>IF($B116="","",SUMPRODUCT(--($B$4:$B116&lt;&gt;"")))</f>
+        <f>IF($B116="","",ROW()-4+1)</f>
       </c>
       <c r="B116" s="17">
         <f>IF('Daily Attendance'!A117="","",'Daily Attendance'!A117)</f>
@@ -29437,7 +29437,7 @@
     </row>
     <row r="117">
       <c r="A117" s="58">
-        <f>IF($B117="","",SUMPRODUCT(--($B$4:$B117&lt;&gt;"")))</f>
+        <f>IF($B117="","",ROW()-4+1)</f>
       </c>
       <c r="B117" s="17">
         <f>IF('Daily Attendance'!A118="","",'Daily Attendance'!A118)</f>
@@ -29472,7 +29472,7 @@
     </row>
     <row r="118">
       <c r="A118" s="58">
-        <f>IF($B118="","",SUMPRODUCT(--($B$4:$B118&lt;&gt;"")))</f>
+        <f>IF($B118="","",ROW()-4+1)</f>
       </c>
       <c r="B118" s="17">
         <f>IF('Daily Attendance'!A119="","",'Daily Attendance'!A119)</f>
@@ -29507,7 +29507,7 @@
     </row>
     <row r="119">
       <c r="A119" s="58">
-        <f>IF($B119="","",SUMPRODUCT(--($B$4:$B119&lt;&gt;"")))</f>
+        <f>IF($B119="","",ROW()-4+1)</f>
       </c>
       <c r="B119" s="17">
         <f>IF('Daily Attendance'!A120="","",'Daily Attendance'!A120)</f>
@@ -29542,7 +29542,7 @@
     </row>
     <row r="120">
       <c r="A120" s="58">
-        <f>IF($B120="","",SUMPRODUCT(--($B$4:$B120&lt;&gt;"")))</f>
+        <f>IF($B120="","",ROW()-4+1)</f>
       </c>
       <c r="B120" s="17">
         <f>IF('Daily Attendance'!A121="","",'Daily Attendance'!A121)</f>
@@ -29577,7 +29577,7 @@
     </row>
     <row r="121">
       <c r="A121" s="58">
-        <f>IF($B121="","",SUMPRODUCT(--($B$4:$B121&lt;&gt;"")))</f>
+        <f>IF($B121="","",ROW()-4+1)</f>
       </c>
       <c r="B121" s="17">
         <f>IF('Daily Attendance'!A122="","",'Daily Attendance'!A122)</f>
@@ -29612,7 +29612,7 @@
     </row>
     <row r="122">
       <c r="A122" s="58">
-        <f>IF($B122="","",SUMPRODUCT(--($B$4:$B122&lt;&gt;"")))</f>
+        <f>IF($B122="","",ROW()-4+1)</f>
       </c>
       <c r="B122" s="17">
         <f>IF('Daily Attendance'!A123="","",'Daily Attendance'!A123)</f>
@@ -29647,7 +29647,7 @@
     </row>
     <row r="123">
       <c r="A123" s="58">
-        <f>IF($B123="","",SUMPRODUCT(--($B$4:$B123&lt;&gt;"")))</f>
+        <f>IF($B123="","",ROW()-4+1)</f>
       </c>
       <c r="B123" s="17">
         <f>IF('Daily Attendance'!A124="","",'Daily Attendance'!A124)</f>
@@ -29682,7 +29682,7 @@
     </row>
     <row r="124">
       <c r="A124" s="58">
-        <f>IF($B124="","",SUMPRODUCT(--($B$4:$B124&lt;&gt;"")))</f>
+        <f>IF($B124="","",ROW()-4+1)</f>
       </c>
       <c r="B124" s="17">
         <f>IF('Daily Attendance'!A125="","",'Daily Attendance'!A125)</f>
@@ -29717,7 +29717,7 @@
     </row>
     <row r="125">
       <c r="A125" s="58">
-        <f>IF($B125="","",SUMPRODUCT(--($B$4:$B125&lt;&gt;"")))</f>
+        <f>IF($B125="","",ROW()-4+1)</f>
       </c>
       <c r="B125" s="17">
         <f>IF('Daily Attendance'!A126="","",'Daily Attendance'!A126)</f>
@@ -29752,7 +29752,7 @@
     </row>
     <row r="126">
       <c r="A126" s="58">
-        <f>IF($B126="","",SUMPRODUCT(--($B$4:$B126&lt;&gt;"")))</f>
+        <f>IF($B126="","",ROW()-4+1)</f>
       </c>
       <c r="B126" s="17">
         <f>IF('Daily Attendance'!A127="","",'Daily Attendance'!A127)</f>
@@ -29787,7 +29787,7 @@
     </row>
     <row r="127">
       <c r="A127" s="58">
-        <f>IF($B127="","",SUMPRODUCT(--($B$4:$B127&lt;&gt;"")))</f>
+        <f>IF($B127="","",ROW()-4+1)</f>
       </c>
       <c r="B127" s="17">
         <f>IF('Daily Attendance'!A128="","",'Daily Attendance'!A128)</f>
@@ -29822,7 +29822,7 @@
     </row>
     <row r="128">
       <c r="A128" s="58">
-        <f>IF($B128="","",SUMPRODUCT(--($B$4:$B128&lt;&gt;"")))</f>
+        <f>IF($B128="","",ROW()-4+1)</f>
       </c>
       <c r="B128" s="17">
         <f>IF('Daily Attendance'!A129="","",'Daily Attendance'!A129)</f>
@@ -29857,7 +29857,7 @@
     </row>
     <row r="129">
       <c r="A129" s="58">
-        <f>IF($B129="","",SUMPRODUCT(--($B$4:$B129&lt;&gt;"")))</f>
+        <f>IF($B129="","",ROW()-4+1)</f>
       </c>
       <c r="B129" s="17">
         <f>IF('Daily Attendance'!A130="","",'Daily Attendance'!A130)</f>
@@ -29892,7 +29892,7 @@
     </row>
     <row r="130">
       <c r="A130" s="58">
-        <f>IF($B130="","",SUMPRODUCT(--($B$4:$B130&lt;&gt;"")))</f>
+        <f>IF($B130="","",ROW()-4+1)</f>
       </c>
       <c r="B130" s="17">
         <f>IF('Daily Attendance'!A131="","",'Daily Attendance'!A131)</f>
@@ -29927,7 +29927,7 @@
     </row>
     <row r="131">
       <c r="A131" s="58">
-        <f>IF($B131="","",SUMPRODUCT(--($B$4:$B131&lt;&gt;"")))</f>
+        <f>IF($B131="","",ROW()-4+1)</f>
       </c>
       <c r="B131" s="17">
         <f>IF('Daily Attendance'!A132="","",'Daily Attendance'!A132)</f>
@@ -29962,7 +29962,7 @@
     </row>
     <row r="132">
       <c r="A132" s="58">
-        <f>IF($B132="","",SUMPRODUCT(--($B$4:$B132&lt;&gt;"")))</f>
+        <f>IF($B132="","",ROW()-4+1)</f>
       </c>
       <c r="B132" s="17">
         <f>IF('Daily Attendance'!A133="","",'Daily Attendance'!A133)</f>
@@ -29997,7 +29997,7 @@
     </row>
     <row r="133">
       <c r="A133" s="58">
-        <f>IF($B133="","",SUMPRODUCT(--($B$4:$B133&lt;&gt;"")))</f>
+        <f>IF($B133="","",ROW()-4+1)</f>
       </c>
       <c r="B133" s="17">
         <f>IF('Daily Attendance'!A134="","",'Daily Attendance'!A134)</f>
@@ -30032,7 +30032,7 @@
     </row>
     <row r="134">
       <c r="A134" s="58">
-        <f>IF($B134="","",SUMPRODUCT(--($B$4:$B134&lt;&gt;"")))</f>
+        <f>IF($B134="","",ROW()-4+1)</f>
       </c>
       <c r="B134" s="17">
         <f>IF('Daily Attendance'!A135="","",'Daily Attendance'!A135)</f>
@@ -30067,7 +30067,7 @@
     </row>
     <row r="135">
       <c r="A135" s="58">
-        <f>IF($B135="","",SUMPRODUCT(--($B$4:$B135&lt;&gt;"")))</f>
+        <f>IF($B135="","",ROW()-4+1)</f>
       </c>
       <c r="B135" s="17">
         <f>IF('Daily Attendance'!A136="","",'Daily Attendance'!A136)</f>
@@ -30102,7 +30102,7 @@
     </row>
     <row r="136">
       <c r="A136" s="58">
-        <f>IF($B136="","",SUMPRODUCT(--($B$4:$B136&lt;&gt;"")))</f>
+        <f>IF($B136="","",ROW()-4+1)</f>
       </c>
       <c r="B136" s="17">
         <f>IF('Daily Attendance'!A137="","",'Daily Attendance'!A137)</f>
@@ -30137,7 +30137,7 @@
     </row>
     <row r="137">
       <c r="A137" s="58">
-        <f>IF($B137="","",SUMPRODUCT(--($B$4:$B137&lt;&gt;"")))</f>
+        <f>IF($B137="","",ROW()-4+1)</f>
       </c>
       <c r="B137" s="17">
         <f>IF('Daily Attendance'!A138="","",'Daily Attendance'!A138)</f>
@@ -30172,7 +30172,7 @@
     </row>
     <row r="138">
       <c r="A138" s="58">
-        <f>IF($B138="","",SUMPRODUCT(--($B$4:$B138&lt;&gt;"")))</f>
+        <f>IF($B138="","",ROW()-4+1)</f>
       </c>
       <c r="B138" s="17">
         <f>IF('Daily Attendance'!A139="","",'Daily Attendance'!A139)</f>
@@ -30207,7 +30207,7 @@
     </row>
     <row r="139">
       <c r="A139" s="58">
-        <f>IF($B139="","",SUMPRODUCT(--($B$4:$B139&lt;&gt;"")))</f>
+        <f>IF($B139="","",ROW()-4+1)</f>
       </c>
       <c r="B139" s="17">
         <f>IF('Daily Attendance'!A140="","",'Daily Attendance'!A140)</f>
@@ -30242,7 +30242,7 @@
     </row>
     <row r="140">
       <c r="A140" s="58">
-        <f>IF($B140="","",SUMPRODUCT(--($B$4:$B140&lt;&gt;"")))</f>
+        <f>IF($B140="","",ROW()-4+1)</f>
       </c>
       <c r="B140" s="17">
         <f>IF('Daily Attendance'!A141="","",'Daily Attendance'!A141)</f>
@@ -30277,7 +30277,7 @@
     </row>
     <row r="141">
       <c r="A141" s="58">
-        <f>IF($B141="","",SUMPRODUCT(--($B$4:$B141&lt;&gt;"")))</f>
+        <f>IF($B141="","",ROW()-4+1)</f>
       </c>
       <c r="B141" s="17">
         <f>IF('Daily Attendance'!A142="","",'Daily Attendance'!A142)</f>
@@ -30312,7 +30312,7 @@
     </row>
     <row r="142">
       <c r="A142" s="58">
-        <f>IF($B142="","",SUMPRODUCT(--($B$4:$B142&lt;&gt;"")))</f>
+        <f>IF($B142="","",ROW()-4+1)</f>
       </c>
       <c r="B142" s="17">
         <f>IF('Daily Attendance'!A143="","",'Daily Attendance'!A143)</f>
@@ -30347,7 +30347,7 @@
     </row>
     <row r="143">
       <c r="A143" s="58">
-        <f>IF($B143="","",SUMPRODUCT(--($B$4:$B143&lt;&gt;"")))</f>
+        <f>IF($B143="","",ROW()-4+1)</f>
       </c>
       <c r="B143" s="17">
         <f>IF('Daily Attendance'!A144="","",'Daily Attendance'!A144)</f>
@@ -30382,7 +30382,7 @@
     </row>
     <row r="144">
       <c r="A144" s="58">
-        <f>IF($B144="","",SUMPRODUCT(--($B$4:$B144&lt;&gt;"")))</f>
+        <f>IF($B144="","",ROW()-4+1)</f>
       </c>
       <c r="B144" s="17">
         <f>IF('Daily Attendance'!A145="","",'Daily Attendance'!A145)</f>
@@ -30417,7 +30417,7 @@
     </row>
     <row r="145">
       <c r="A145" s="58">
-        <f>IF($B145="","",SUMPRODUCT(--($B$4:$B145&lt;&gt;"")))</f>
+        <f>IF($B145="","",ROW()-4+1)</f>
       </c>
       <c r="B145" s="17">
         <f>IF('Daily Attendance'!A146="","",'Daily Attendance'!A146)</f>
@@ -30452,7 +30452,7 @@
     </row>
     <row r="146">
       <c r="A146" s="58">
-        <f>IF($B146="","",SUMPRODUCT(--($B$4:$B146&lt;&gt;"")))</f>
+        <f>IF($B146="","",ROW()-4+1)</f>
       </c>
       <c r="B146" s="17">
         <f>IF('Daily Attendance'!A147="","",'Daily Attendance'!A147)</f>
@@ -30487,7 +30487,7 @@
     </row>
     <row r="147">
       <c r="A147" s="58">
-        <f>IF($B147="","",SUMPRODUCT(--($B$4:$B147&lt;&gt;"")))</f>
+        <f>IF($B147="","",ROW()-4+1)</f>
       </c>
       <c r="B147" s="17">
         <f>IF('Daily Attendance'!A148="","",'Daily Attendance'!A148)</f>
@@ -30522,7 +30522,7 @@
     </row>
     <row r="148">
       <c r="A148" s="58">
-        <f>IF($B148="","",SUMPRODUCT(--($B$4:$B148&lt;&gt;"")))</f>
+        <f>IF($B148="","",ROW()-4+1)</f>
       </c>
       <c r="B148" s="17">
         <f>IF('Daily Attendance'!A149="","",'Daily Attendance'!A149)</f>
@@ -30557,7 +30557,7 @@
     </row>
     <row r="149">
       <c r="A149" s="58">
-        <f>IF($B149="","",SUMPRODUCT(--($B$4:$B149&lt;&gt;"")))</f>
+        <f>IF($B149="","",ROW()-4+1)</f>
       </c>
       <c r="B149" s="17">
         <f>IF('Daily Attendance'!A150="","",'Daily Attendance'!A150)</f>
@@ -30592,7 +30592,7 @@
     </row>
     <row r="150">
       <c r="A150" s="58">
-        <f>IF($B150="","",SUMPRODUCT(--($B$4:$B150&lt;&gt;"")))</f>
+        <f>IF($B150="","",ROW()-4+1)</f>
       </c>
       <c r="B150" s="17">
         <f>IF('Daily Attendance'!A151="","",'Daily Attendance'!A151)</f>
@@ -30627,7 +30627,7 @@
     </row>
     <row r="151">
       <c r="A151" s="58">
-        <f>IF($B151="","",SUMPRODUCT(--($B$4:$B151&lt;&gt;"")))</f>
+        <f>IF($B151="","",ROW()-4+1)</f>
       </c>
       <c r="B151" s="17">
         <f>IF('Daily Attendance'!A152="","",'Daily Attendance'!A152)</f>
@@ -30662,7 +30662,7 @@
     </row>
     <row r="152">
       <c r="A152" s="58">
-        <f>IF($B152="","",SUMPRODUCT(--($B$4:$B152&lt;&gt;"")))</f>
+        <f>IF($B152="","",ROW()-4+1)</f>
       </c>
       <c r="B152" s="17">
         <f>IF('Daily Attendance'!A153="","",'Daily Attendance'!A153)</f>
@@ -30697,7 +30697,7 @@
     </row>
     <row r="153">
       <c r="A153" s="58">
-        <f>IF($B153="","",SUMPRODUCT(--($B$4:$B153&lt;&gt;"")))</f>
+        <f>IF($B153="","",ROW()-4+1)</f>
       </c>
       <c r="B153" s="17">
         <f>IF('Daily Attendance'!A154="","",'Daily Attendance'!A154)</f>
@@ -30732,7 +30732,7 @@
     </row>
     <row r="154">
       <c r="A154" s="58">
-        <f>IF($B154="","",SUMPRODUCT(--($B$4:$B154&lt;&gt;"")))</f>
+        <f>IF($B154="","",ROW()-4+1)</f>
       </c>
       <c r="B154" s="17">
         <f>IF('Daily Attendance'!A155="","",'Daily Attendance'!A155)</f>
@@ -30767,7 +30767,7 @@
     </row>
     <row r="155">
       <c r="A155" s="58">
-        <f>IF($B155="","",SUMPRODUCT(--($B$4:$B155&lt;&gt;"")))</f>
+        <f>IF($B155="","",ROW()-4+1)</f>
       </c>
       <c r="B155" s="17">
         <f>IF('Daily Attendance'!A156="","",'Daily Attendance'!A156)</f>
@@ -30802,7 +30802,7 @@
     </row>
     <row r="156">
       <c r="A156" s="58">
-        <f>IF($B156="","",SUMPRODUCT(--($B$4:$B156&lt;&gt;"")))</f>
+        <f>IF($B156="","",ROW()-4+1)</f>
       </c>
       <c r="B156" s="17">
         <f>IF('Daily Attendance'!A157="","",'Daily Attendance'!A157)</f>
@@ -30837,7 +30837,7 @@
     </row>
     <row r="157">
       <c r="A157" s="58">
-        <f>IF($B157="","",SUMPRODUCT(--($B$4:$B157&lt;&gt;"")))</f>
+        <f>IF($B157="","",ROW()-4+1)</f>
       </c>
       <c r="B157" s="17">
         <f>IF('Daily Attendance'!A158="","",'Daily Attendance'!A158)</f>
@@ -30872,7 +30872,7 @@
     </row>
     <row r="158">
       <c r="A158" s="58">
-        <f>IF($B158="","",SUMPRODUCT(--($B$4:$B158&lt;&gt;"")))</f>
+        <f>IF($B158="","",ROW()-4+1)</f>
       </c>
       <c r="B158" s="17">
         <f>IF('Daily Attendance'!A159="","",'Daily Attendance'!A159)</f>
@@ -30907,7 +30907,7 @@
     </row>
     <row r="159">
       <c r="A159" s="58">
-        <f>IF($B159="","",SUMPRODUCT(--($B$4:$B159&lt;&gt;"")))</f>
+        <f>IF($B159="","",ROW()-4+1)</f>
       </c>
       <c r="B159" s="17">
         <f>IF('Daily Attendance'!A160="","",'Daily Attendance'!A160)</f>
@@ -30942,7 +30942,7 @@
     </row>
     <row r="160">
       <c r="A160" s="58">
-        <f>IF($B160="","",SUMPRODUCT(--($B$4:$B160&lt;&gt;"")))</f>
+        <f>IF($B160="","",ROW()-4+1)</f>
       </c>
       <c r="B160" s="17">
         <f>IF('Daily Attendance'!A161="","",'Daily Attendance'!A161)</f>
@@ -30977,7 +30977,7 @@
     </row>
     <row r="161">
       <c r="A161" s="58">
-        <f>IF($B161="","",SUMPRODUCT(--($B$4:$B161&lt;&gt;"")))</f>
+        <f>IF($B161="","",ROW()-4+1)</f>
       </c>
       <c r="B161" s="17">
         <f>IF('Daily Attendance'!A162="","",'Daily Attendance'!A162)</f>
@@ -31012,7 +31012,7 @@
     </row>
     <row r="162">
       <c r="A162" s="58">
-        <f>IF($B162="","",SUMPRODUCT(--($B$4:$B162&lt;&gt;"")))</f>
+        <f>IF($B162="","",ROW()-4+1)</f>
       </c>
       <c r="B162" s="17">
         <f>IF('Daily Attendance'!A163="","",'Daily Attendance'!A163)</f>
@@ -31047,7 +31047,7 @@
     </row>
     <row r="163">
       <c r="A163" s="58">
-        <f>IF($B163="","",SUMPRODUCT(--($B$4:$B163&lt;&gt;"")))</f>
+        <f>IF($B163="","",ROW()-4+1)</f>
       </c>
       <c r="B163" s="17">
         <f>IF('Daily Attendance'!A164="","",'Daily Attendance'!A164)</f>

</xml_diff>